<commit_message>
Add descent-closed atom quotient audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rbc19d166628944a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd6937e7bca824baa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -951,7 +951,7 @@
         <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>Atom descent closure, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D42" t="str">
         <x:v>Executable audit</x:v>

</xml_diff>

<commit_message>
Record closure derivation provenance
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd6937e7bca824baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R421df79a25b041a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -407,7 +407,7 @@
         <x:v>Route finite intervals only after exact local-minimality evidence.</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Single-pair closure counters expose failures and max depth.</x:v>
+        <x:v>Single-pair closure counters expose failures and max depth; derivation rows now record the first seed/forward/inverse proof of each generated relation edge.</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>Proof hygiene</x:v>

</xml_diff>

<commit_message>
Add extra corridor detector factors
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R421df79a25b041a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rc9bf6fae96664a64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1223,7 +1223,7 @@
         <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D58" t="str">
         <x:v>Open theorem target</x:v>
@@ -1240,7 +1240,7 @@
         <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Helper, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>Executable audit</x:v>

</xml_diff>

<commit_message>
Add congruence chain rack assembly
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rc9bf6fae96664a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R934ff18edf5b4932"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -356,7 +356,7 @@
         <x:v>Local detectors compose down congruence chain.</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Cover/local extraction implemented.</x:v>
+        <x:v>Cover/local extraction implemented; assemble_congruence_chain_rack iterates Q_i=Q_{i+1} x A_{G_i} and records |Q_i|=|Q_{i+1}|*2*|G_i|^2 without an n parameter.</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>Executable audit</x:v>

</xml_diff>

<commit_message>
Record elementary kernel corridor counters
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R934ff18edf5b4932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rc2e96cdb29f94bb8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1308,7 +1308,7 @@
         <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; elementary kernel-pair closure gate added.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D63" t="str">
         <x:v>Candidate audit</x:v>

</xml_diff>

<commit_message>
Add normalized law sequence gate
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rc2e96cdb29f94bb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rc312a2182ea04de0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -747,7 +747,7 @@
         <x:v>Audit exponent-law braid shortcut.</x:v>
       </x:c>
       <x:c r="C30" t="str">
-        <x:v>Pure-power shortcut ruled insufficient.</x:v>
+        <x:v>Pure-power shortcut ruled insufficient; normalized_law_sequence_gate records the order-prefix law condition and prefix audit helper.</x:v>
       </x:c>
       <x:c r="D30" t="str">
         <x:v>Gap clarified</x:v>

</xml_diff>

<commit_message>
Add known branch detector certificates
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rc312a2182ea04de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R76d9f40b6f684a5b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1070,7 +1070,7 @@
         <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D49" t="str">
         <x:v>Symbolic branch proof</x:v>
@@ -1206,7 +1206,7 @@
         <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Router now splits closed product finite-G branches from product/corridor bottlenecks.</x:v>
+        <x:v>Router now splits closed product finite-G branches from product/corridor bottlenecks and records explicit known-branch detector reason/order/factor size.</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>Reduction ledger</x:v>

</xml_diff>

<commit_message>
Record closed product detector certificates
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R76d9f40b6f684a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R5d56f55e3d574920"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1206,7 +1206,7 @@
         <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Router now splits closed product finite-G branches from product/corridor bottlenecks and records explicit known-branch detector reason/order/factor size.</x:v>
+        <x:v>Router now records explicit known-branch and closed-product detector reason/order/factor size, with fibre2 affine product rows marked as delegated.</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>Reduction ledger</x:v>
@@ -1359,7 +1359,7 @@
         <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>H_prod explicit; coboundaries telescope.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector certificates added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D66" t="str">
         <x:v>Executable audit</x:v>
@@ -1478,7 +1478,7 @@
         <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity and pairwise branch is C3-detected.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate orders are exposed.</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>Reduction criterion</x:v>

</xml_diff>

<commit_message>
Attach product detector group objects
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R5d56f55e3d574920"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rdcbd2b0f1bc64462"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1206,7 +1206,7 @@
         <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Router now records explicit known-branch and closed-product detector reason/order/factor size, with fibre2 affine product rows marked as delegated.</x:v>
+        <x:v>Router now records explicit known-branch and closed-product detector group/order/factor size, with fibre2 affine product rows marked as delegated.</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>Reduction ledger</x:v>
@@ -1359,7 +1359,7 @@
         <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector certificates added to bottleneck summary.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D66" t="str">
         <x:v>Executable audit</x:v>
@@ -1478,7 +1478,7 @@
         <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate orders are exposed.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>Reduction criterion</x:v>

</xml_diff>

<commit_message>
Expose closed local detector groups
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rdcbd2b0f1bc64462"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R79048586ebc343ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1206,7 +1206,7 @@
         <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Router now records explicit known-branch and closed-product detector group/order/factor size, with fibre2 affine product rows marked as delegated.</x:v>
+        <x:v>Router now records explicit known/product detector groups and merged closed_detector_groups/closed_detector_gaps handoff.</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>Reduction ledger</x:v>

</xml_diff>

<commit_message>
Add bi-free endpoint factorization
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R79048586ebc343ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Re65bd8d270dd4744"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -356,7 +356,7 @@
         <x:v>Local detectors compose down congruence chain.</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Cover/local extraction implemented; assemble_congruence_chain_rack iterates Q_i=Q_{i+1} x A_{G_i} and records |Q_i|=|Q_{i+1}|*2*|G_i|^2 without an n parameter.</x:v>
+        <x:v>Cover/local extraction implemented; closed_local_detector_chain requires one fixed product group per closed interval before assemble_congruence_chain_rack builds Q_i=Q_{i+1} x A_{G_i}.</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>Executable audit</x:v>
@@ -1206,7 +1206,7 @@
         <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Router now records explicit known/product detector groups and merged closed_detector_groups/closed_detector_gaps handoff.</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>Reduction ledger</x:v>
@@ -1234,499 +1234,516 @@
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/bifree_corridor_endpoint_factorization.md proves factorwise endpoint witnesses in H_s combine in H(pi,Q) and identity product longitudes kill faithful endpoint readouts.</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove the endpoint longitudinalization lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D68" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D72" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="48" customHeight="1">
+      <x:c r="A88" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B87" t="str">
+      <x:c r="B88" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C87" t="str">
+      <x:c r="C88" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D87" t="str">
+      <x:c r="D88" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E87" t="str">
+      <x:c r="E88" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D87">
+  <x:conditionalFormatting sqref="D2:D88">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add endpoint expression audits
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Re65bd8d270dd4744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R58859fc0fd984b73"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1240,7 +1240,7 @@
         <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>proofs/bifree_corridor_endpoint_factorization.md proves factorwise endpoint witnesses in H_s combine in H(pi,Q) and identity product longitudes kill faithful endpoint readouts.</x:v>
+        <x:v>Proof note plus endpoint_*_longitude_expression_audit helpers build literal product witnesses in V_beta(H(pi,Q)) from displayed factor expressions.</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>Assembly lemma</x:v>

</xml_diff>

<commit_message>
Add endpoint readout audits
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R58859fc0fd984b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R0e5fe84263e94cd8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1240,7 +1240,7 @@
         <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Proof note plus endpoint_*_longitude_expression_audit helpers build literal product witnesses in V_beta(H(pi,Q)) from displayed factor expressions.</x:v>
+        <x:v>Proof note plus endpoint expression/readout helpers build literal product witnesses and verify the identity-endpoint faithful-readout gate.</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>Assembly lemma</x:v>

</xml_diff>

<commit_message>
Add endpoint residual action audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R0e5fe84263e94cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R4279386df0324bb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1240,7 +1240,7 @@
         <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Proof note plus endpoint expression/readout helpers build literal product witnesses and verify the identity-endpoint faithful-readout gate.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims.</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>Assembly lemma</x:v>

</xml_diff>

<commit_message>
Add Artin-defect endpoint sieve
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R4279386df0324bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Re0f34bff0bf546e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1240,510 +1240,527 @@
         <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Prove the endpoint longitudinalization lemma for every target interval.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D69" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D74" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="48" customHeight="1">
+      <x:c r="A89" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B88" t="str">
+      <x:c r="B89" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C88" t="str">
+      <x:c r="C89" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D88" t="str">
+      <x:c r="D89" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E88" t="str">
+      <x:c r="E89" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D88">
+  <x:conditionalFormatting sqref="D2:D89">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add Artin detector-lift criterion
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Re0f34bff0bf546e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R435e2446c6794771"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1268,499 +1268,516 @@
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D70" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D74" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="48" customHeight="1">
+      <x:c r="A90" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B89" t="str">
+      <x:c r="B90" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C89" t="str">
+      <x:c r="C90" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D89" t="str">
+      <x:c r="D90" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E89" t="str">
+      <x:c r="E90" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D89">
+  <x:conditionalFormatting sqref="D2:D90">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Close atom-inner detector-lift rows
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R435e2446c6794771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd2b2c40534d2413d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1285,499 +1285,516 @@
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D71" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="48" customHeight="1">
+      <x:c r="A91" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B90" t="str">
+      <x:c r="B91" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C90" t="str">
+      <x:c r="C91" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D90" t="str">
+      <x:c r="D91" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E90" t="str">
+      <x:c r="E91" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D90">
+  <x:conditionalFormatting sqref="D2:D91">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add Green first-output defect criterion
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd2b2c40534d2413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Ra6b1a7a2ebab43f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1302,499 +1302,516 @@
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove transported Schutzenberger defect endpoints D_C(beta) lie in V_beta(Sch(C)); handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D72" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="48" customHeight="1">
+      <x:c r="A92" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B91" t="str">
+      <x:c r="B92" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C91" t="str">
+      <x:c r="C92" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D91" t="str">
+      <x:c r="D92" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E91" t="str">
+      <x:c r="E92" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D91">
+  <x:conditionalFormatting sqref="D2:D92">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add Green defect-kernel quotient criterion
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Ra6b1a7a2ebab43f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R72f324c95c104cda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1314,504 +1314,521 @@
         <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Prove transported Schutzenberger defect endpoints D_C(beta) lie in V_beta(Sch(C)); handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="48" customHeight="1">
+      <x:c r="A93" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B92" t="str">
+      <x:c r="B93" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C92" t="str">
+      <x:c r="C93" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D92" t="str">
+      <x:c r="D93" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E92" t="str">
+      <x:c r="E93" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D92">
+  <x:conditionalFormatting sqref="D2:D93">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add Green defect potential coboundary criterion
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R72f324c95c104cda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R37be74c4a5bb4755"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1336,499 +1336,516 @@
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D74" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="48" customHeight="1">
+      <x:c r="A94" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B93" t="str">
+      <x:c r="B94" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C93" t="str">
+      <x:c r="C94" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D93" t="str">
+      <x:c r="D94" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E93" t="str">
+      <x:c r="E94" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D93">
+  <x:conditionalFormatting sqref="D2:D94">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add Artin defect abelianization barrier
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R37be74c4a5bb4755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R4c062ac343f94e4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1353,499 +1353,516 @@
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="48" customHeight="1">
+      <x:c r="A95" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B94" t="str">
+      <x:c r="B95" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C94" t="str">
+      <x:c r="C95" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D94" t="str">
+      <x:c r="D95" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E94" t="str">
+      <x:c r="E95" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D94">
+  <x:conditionalFormatting sqref="D2:D95">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add Green defect abelianization split
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R4c062ac343f94e4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R6614645c118b4940"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1370,499 +1370,516 @@
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="48" customHeight="1">
+      <x:c r="A96" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B95" t="str">
+      <x:c r="B96" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C95" t="str">
+      <x:c r="C96" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D95" t="str">
+      <x:c r="D96" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E95" t="str">
+      <x:c r="E96" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D95">
+  <x:conditionalFormatting sqref="D2:D96">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add abelian longitude image criterion
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R6614645c118b4940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R7d03dc297e914aab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1387,499 +1387,516 @@
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="48" customHeight="1">
+      <x:c r="A97" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B96" t="str">
+      <x:c r="B97" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C96" t="str">
+      <x:c r="C97" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D96" t="str">
+      <x:c r="D97" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E96" t="str">
+      <x:c r="E97" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D96">
+  <x:conditionalFormatting sqref="D2:D97">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add balanced Green gauge decomposition
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R7d03dc297e914aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R43e359224233459f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1404,499 +1404,516 @@
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="48" customHeight="1">
+      <x:c r="A98" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B97" t="str">
+      <x:c r="B98" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C97" t="str">
+      <x:c r="C98" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D97" t="str">
+      <x:c r="D98" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E97" t="str">
+      <x:c r="E98" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D97">
+  <x:conditionalFormatting sqref="D2:D98">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add terminal and principal gauge criteria
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R43e359224233459f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rcaeb9a1bec3047c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1421,499 +1421,533 @@
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Open</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
+        <x:v>Master theorem</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>Prove detection or realize escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="48" customHeight="1">
+      <x:c r="A99" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="48" customHeight="1">
+      <x:c r="A100" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B98" t="str">
+      <x:c r="B100" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C98" t="str">
+      <x:c r="C100" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D98" t="str">
+      <x:c r="D100" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E98" t="str">
+      <x:c r="E100" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D98">
+  <x:conditionalFormatting sqref="D2:D100">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add transport-state rackification detector
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rcaeb9a1bec3047c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R75adb587fe5d4201"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1455,499 +1455,516 @@
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="48" customHeight="1">
+      <x:c r="A101" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B100" t="str">
+      <x:c r="B101" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C100" t="str">
+      <x:c r="C101" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D100" t="str">
+      <x:c r="D101" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E100" t="str">
+      <x:c r="E101" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D100">
+  <x:conditionalFormatting sqref="D2:D101">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add descent-separation reduction gates
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R75adb587fe5d4201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rdac8e6ce90e44860"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1472,499 +1472,550 @@
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Open</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
+        <x:v>Known branches</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>Branch list recorded in proof log.</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>Bookkept</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="48" customHeight="1">
+      <x:c r="A102" t="str">
+        <x:v>Master theorem</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>Prove detection or realize escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="48" customHeight="1">
+      <x:c r="A103" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="48" customHeight="1">
+      <x:c r="A104" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B101" t="str">
+      <x:c r="B104" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C101" t="str">
+      <x:c r="C104" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D101" t="str">
+      <x:c r="D104" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E101" t="str">
+      <x:c r="E104" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D101">
+  <x:conditionalFormatting sqref="D2:D104">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add elementary continuation closure gate
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rdac8e6ce90e44860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R50a62025324c4acb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1489,533 +1489,550 @@
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="48" customHeight="1">
+      <x:c r="A105" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B104" t="str">
+      <x:c r="B105" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C104" t="str">
+      <x:c r="C105" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D104" t="str">
+      <x:c r="D105" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E104" t="str">
+      <x:c r="E105" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D104">
+  <x:conditionalFormatting sqref="D2:D105">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add universal continuation derivation certificate
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R50a62025324c4acb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R7952dcad5ec3454a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1506,533 +1506,550 @@
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="48" customHeight="1">
+      <x:c r="A106" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B105" t="str">
+      <x:c r="B106" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C105" t="str">
+      <x:c r="C106" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D105" t="str">
+      <x:c r="D106" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E105" t="str">
+      <x:c r="E106" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D105">
+  <x:conditionalFormatting sqref="D2:D106">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add continuation readout propagation criterion
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R7952dcad5ec3454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb8184d06d67a46e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1523,533 +1523,550 @@
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="48" customHeight="1">
+      <x:c r="A107" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B106" t="str">
+      <x:c r="B107" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C106" t="str">
+      <x:c r="C107" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D106" t="str">
+      <x:c r="D107" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E106" t="str">
+      <x:c r="E107" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D106">
+  <x:conditionalFormatting sqref="D2:D107">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add readout kernel admissibility criterion
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb8184d06d67a46e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Ra6fd894927b5465e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1540,533 +1540,550 @@
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="48" customHeight="1">
+      <x:c r="A108" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B107" t="str">
+      <x:c r="B108" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C107" t="str">
+      <x:c r="C108" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D107" t="str">
+      <x:c r="D108" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E107" t="str">
+      <x:c r="E108" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D107">
+  <x:conditionalFormatting sqref="D2:D108">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add readout descent separation certificate
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Ra6fd894927b5465e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R38f753a002a9433c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1557,533 +1557,550 @@
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="48" customHeight="1">
+      <x:c r="A109" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B108" t="str">
+      <x:c r="B109" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C108" t="str">
+      <x:c r="C109" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D108" t="str">
+      <x:c r="D109" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E108" t="str">
+      <x:c r="E109" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D108">
+  <x:conditionalFormatting sqref="D2:D109">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add readout kernel quotient interval
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R38f753a002a9433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Re03b65ca30e447f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1574,533 +1574,550 @@
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="48" customHeight="1">
+      <x:c r="A110" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B109" t="str">
+      <x:c r="B110" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C109" t="str">
+      <x:c r="C110" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D109" t="str">
+      <x:c r="D110" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E109" t="str">
+      <x:c r="E110" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D109">
+  <x:conditionalFormatting sqref="D2:D110">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add product readout kernel assembly
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Re03b65ca30e447f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R819b789376154b82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1591,533 +1591,550 @@
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="48" customHeight="1">
+      <x:c r="A111" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B110" t="str">
+      <x:c r="B111" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C110" t="str">
+      <x:c r="C111" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D110" t="str">
+      <x:c r="D111" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E110" t="str">
+      <x:c r="E111" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D110">
+  <x:conditionalFormatting sqref="D2:D111">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add product descent separation audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R819b789376154b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R5d114096cb6e4366"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1608,533 +1608,550 @@
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="48" customHeight="1">
+      <x:c r="A112" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B111" t="str">
+      <x:c r="B112" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C111" t="str">
+      <x:c r="C112" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D111" t="str">
+      <x:c r="D112" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E111" t="str">
+      <x:c r="E112" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D111">
+  <x:conditionalFormatting sqref="D2:D112">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add readout seed saturation audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R5d114096cb6e4366"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R04deed89d97e4a08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1625,533 +1625,550 @@
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="48" customHeight="1">
+      <x:c r="A113" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B112" t="str">
+      <x:c r="B113" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C112" t="str">
+      <x:c r="C113" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D112" t="str">
+      <x:c r="D113" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E112" t="str">
+      <x:c r="E113" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D112">
+  <x:conditionalFormatting sqref="D2:D113">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add local-minimal seed saturation dichotomy
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R04deed89d97e4a08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R684cec888825452f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1642,533 +1642,550 @@
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="48" customHeight="1">
+      <x:c r="A114" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B113" t="str">
+      <x:c r="B114" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C113" t="str">
+      <x:c r="C114" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D113" t="str">
+      <x:c r="D114" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E113" t="str">
+      <x:c r="E114" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D113">
+  <x:conditionalFormatting sqref="D2:D114">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add lost-edge external routing ledger
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R684cec888825452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R7813987bf3784b06"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1659,533 +1659,550 @@
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="48" customHeight="1">
+      <x:c r="A115" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B114" t="str">
+      <x:c r="B115" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C114" t="str">
+      <x:c r="C115" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D114" t="str">
+      <x:c r="D115" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E114" t="str">
+      <x:c r="E115" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D114">
+  <x:conditionalFormatting sqref="D2:D115">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add continuation endpoint obstruction notes
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R7813987bf3784b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb36ab07f5fa944ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1676,533 +1676,567 @@
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open theorem</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Sharper open theorem</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Prove every residual unit-continuation endpoint lies in V_beta(U_cont), or upgrade such a failure to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Open</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
+        <x:v>Master theorem</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E115" t="str">
+        <x:v>Prove detection or realize escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="48" customHeight="1">
+      <x:c r="A116" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="48" customHeight="1">
+      <x:c r="A117" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B115" t="str">
+      <x:c r="B117" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C115" t="str">
+      <x:c r="C117" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D115" t="str">
+      <x:c r="D117" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E115" t="str">
+      <x:c r="E117" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D115">
+  <x:conditionalFormatting sqref="D2:D117">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add unit continuation abelian lift
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb36ab07f5fa944ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rbb31f3504d674a1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1744,499 +1744,516 @@
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E117" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="48" customHeight="1">
+      <x:c r="A118" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B117" t="str">
+      <x:c r="B118" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C117" t="str">
+      <x:c r="C118" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D117" t="str">
+      <x:c r="D118" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E117" t="str">
+      <x:c r="E118" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D117">
+  <x:conditionalFormatting sqref="D2:D118">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add mixed-unit continuation reductions
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rbb31f3504d674a1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R2f01de3614a6419f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1744,516 +1744,550 @@
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Sharper open theorem</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Prove no mixed-unit universal-continuation context recovery in a local-minimal bottleneck, or extract normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Open</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
+        <x:v>Master theorem</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>Prove detection or realize escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="48" customHeight="1">
+      <x:c r="A119" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="48" customHeight="1">
+      <x:c r="A120" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B118" t="str">
+      <x:c r="B120" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C118" t="str">
+      <x:c r="C120" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D118" t="str">
+      <x:c r="D120" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E118" t="str">
+      <x:c r="E120" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D118">
+  <x:conditionalFormatting sqref="D2:D120">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add mixed-unit companion separation audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R2f01de3614a6419f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R2045bb7a98074e3a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1761,533 +1761,550 @@
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D115" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="48" customHeight="1">
+      <x:c r="A121" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B120" t="str">
+      <x:c r="B121" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C120" t="str">
+      <x:c r="C121" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D120" t="str">
+      <x:c r="D121" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E120" t="str">
+      <x:c r="E121" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D120">
+  <x:conditionalFormatting sqref="D2:D121">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add rank-profile collapse audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R2045bb7a98074e3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R2e260ab6f6774a99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1778,533 +1778,550 @@
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Sharper open theorem</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Classify constant-section triangular YBE rows in the local-minimal bottleneck branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D115" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="48" customHeight="1">
+      <x:c r="A122" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B121" t="str">
+      <x:c r="B122" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C121" t="str">
+      <x:c r="C122" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D121" t="str">
+      <x:c r="D122" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E121" t="str">
+      <x:c r="E122" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D121">
+  <x:conditionalFormatting sqref="D2:D122">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add triangular bundle partition audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R2e260ab6f6774a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R0649db6222f644f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1795,533 +1795,550 @@
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Sharper open theorem</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Classify triangular bundle holonomy or upgrade a bundle holonomy cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D115" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="48" customHeight="1">
+      <x:c r="A123" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B122" t="str">
+      <x:c r="B123" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C122" t="str">
+      <x:c r="C123" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D122" t="str">
+      <x:c r="D123" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E122" t="str">
+      <x:c r="E123" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D122">
+  <x:conditionalFormatting sqref="D2:D123">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add constant-column collapse audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R0649db6222f644f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R1049a5316b95410a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1812,533 +1812,567 @@
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Sharper open theorem</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Longitudinalize triangular recovery holonomy, or upgrade a recovery cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Final triangular target</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove the Latin-unit triangular longitude theorem for U_triangle, or upgrade a Latin-unit endpoint miss to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Open</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
+        <x:v>Master theorem</x:v>
+      </x:c>
+      <x:c r="B123" t="str">
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>Prove detection or realize escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="48" customHeight="1">
+      <x:c r="A124" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B124" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="48" customHeight="1">
+      <x:c r="A125" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B123" t="str">
+      <x:c r="B125" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C123" t="str">
+      <x:c r="C125" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D123" t="str">
+      <x:c r="D125" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E123" t="str">
+      <x:c r="E125" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D123">
+  <x:conditionalFormatting sqref="D2:D125">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add Latin triangular YBE split audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R1049a5316b95410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd57a6d4c38ce4608"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1846,533 +1846,550 @@
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Sharper triangular target</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Route alpha through product/permutation holonomy and prove companion-shear endpoints lie in V_beta(U_shear), or upgrade a shear miss to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B125" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="48" customHeight="1">
+      <x:c r="A126" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B125" t="str">
+      <x:c r="B126" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C125" t="str">
+      <x:c r="C126" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D125" t="str">
+      <x:c r="D126" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E125" t="str">
+      <x:c r="E126" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D125">
+  <x:conditionalFormatting sqref="D2:D126">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add kink predecessor Latin cancellation
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd57a6d4c38ce4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R11d182f6470a45fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1863,533 +1863,567 @@
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Conditional local closure</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>With prior branch reductions accepted, the bi-free universal-corridor lower-row obstruction is eliminated.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Open</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D115" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
+        <x:v>Master theorem</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>Prove detection or realize escape.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="48" customHeight="1">
+      <x:c r="A127" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="48" customHeight="1">
+      <x:c r="A128" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B126" t="str">
+      <x:c r="B128" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C126" t="str">
+      <x:c r="C128" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D126" t="str">
+      <x:c r="D128" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E126" t="str">
+      <x:c r="E128" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D126">
+  <x:conditionalFormatting sqref="D2:D128">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Assemble master local positive closure
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R11d182f6470a45fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R564550cb233840d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1897,533 +1897,550 @@
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md cites the branch notes and proves Lambda_H=1 implies Delta=1 for each local-minimal interval.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Candidate A proof</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Run final proof-critic audit for finite-search leakage, semisplit handling, n-independence, and chain induction before marking the global goal complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D127" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="48" customHeight="1">
+      <x:c r="A129" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B128" t="str">
+      <x:c r="B129" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C128" t="str">
+      <x:c r="C129" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D128" t="str">
+      <x:c r="D129" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E128" t="str">
+      <x:c r="E129" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D128">
+  <x:conditionalFormatting sqref="D2:D129">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add final completion audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R564550cb233840d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb1035bd676994a96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1909,538 +1909,555 @@
         <x:v>Candidate A proof</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Run final proof-critic audit for finite-search leakage, semisplit handling, n-independence, and chain induction before marking the global goal complete.</x:v>
+        <x:v>Audit finite-search leakage, semisplit handling, n-independence, endpoint faithfulness, and chain induction against proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Final completion audit</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Check the assembled A-route against the explicit Sawin requirements and record the failed external proof-critic attempt.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md audits quotient/residual setup, sharp obstruction, congruence-chain induction, local-minimality gates, fixed detector independence from n, and non-use of finite search; Chrome/Browser proof critic failed before tab discovery.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Internal completion audit</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Obtain external GPT-5.5 Pro or human referee review if browser access becomes available; otherwise keep the audit artifact with the branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D115" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D125" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D128" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="48" customHeight="1">
+      <x:c r="A130" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B129" t="str">
+      <x:c r="B130" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C129" t="str">
+      <x:c r="C130" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D129" t="str">
+      <x:c r="D130" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E129" t="str">
+      <x:c r="E130" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D129">
+  <x:conditionalFormatting sqref="D2:D130">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Record proof critic gap audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb1035bd676994a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Ree42badb4fe048dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1716,13 +1716,13 @@
         <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records that transport-rack closure is proved and descent separation remains open.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Open theorem</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove universal continuation visibility or extract a normalized-law B seed from a non-separated row.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
@@ -1736,10 +1736,10 @@
         <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Sharper open theorem</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove every residual unit-continuation endpoint lies in V_beta(U_cont), or upgrade such a failure to normalized laws.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
@@ -1753,10 +1753,10 @@
         <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Sharper open theorem</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove no mixed-unit universal-continuation context recovery in a local-minimal bottleneck, or extract normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
@@ -1787,10 +1787,10 @@
         <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Sharper open theorem</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Classify constant-section triangular YBE rows in the local-minimal bottleneck branch.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
@@ -1804,10 +1804,10 @@
         <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Sharper open theorem</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Classify triangular bundle holonomy or upgrade a bundle holonomy cycle to normalized laws.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
@@ -1821,10 +1821,10 @@
         <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Sharper open theorem</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Longitudinalize triangular recovery holonomy, or upgrade a recovery cycle to normalized laws.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
@@ -1838,10 +1838,10 @@
         <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Final triangular target</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Prove the Latin-unit triangular longitude theorem for U_triangle, or upgrade a Latin-unit endpoint miss to normalized laws.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
@@ -1855,10 +1855,10 @@
         <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Sharper triangular target</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Route alpha through product/permutation holonomy and prove companion-shear endpoints lie in V_beta(U_shear), or upgrade a shear miss to normalized laws.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
@@ -1889,10 +1889,10 @@
         <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Conditional local closure</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>With prior branch reductions accepted, the bi-free universal-corridor lower-row obstruction is eliminated.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
@@ -1903,561 +1903,578 @@
         <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md cites the branch notes and proves Lambda_H=1 implies Delta=1 for each local-minimal interval.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Candidate A proof</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Audit finite-search leakage, semisplit handling, n-independence, endpoint faithfulness, and chain induction against proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Final completion audit</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Check the assembled A-route against the explicit Sawin requirements and record the failed external proof-critic attempt.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/final_completion_audit.md audits quotient/residual setup, sharp obstruction, congruence-chain induction, local-minimality gates, fixed detector independence from n, and non-use of finite search; Chrome/Browser proof critic failed before tab discovery.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Internal completion audit</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Obtain external GPT-5.5 Pro or human referee review if browser access becomes available; otherwise keep the audit artifact with the branch.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D115" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D125" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D126" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D129" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="48" customHeight="1">
+      <x:c r="A131" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B130" t="str">
+      <x:c r="B131" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C130" t="str">
+      <x:c r="C131" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D130" t="str">
+      <x:c r="D131" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E130" t="str">
+      <x:c r="E131" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D130">
+  <x:conditionalFormatting sqref="D2:D131">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add descent endpoint repair contract
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Ree42badb4fe048dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb0c88d3aabd94892"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1931,550 +1931,567 @@
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D125" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D126" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D127" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D130" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="48" customHeight="1">
+      <x:c r="A132" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B131" t="str">
+      <x:c r="B132" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C131" t="str">
+      <x:c r="C132" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D131" t="str">
+      <x:c r="D132" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E131" t="str">
+      <x:c r="E132" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D131">
+  <x:conditionalFormatting sqref="D2:D132">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add executable repair contract audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rb0c88d3aabd94892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd0f82e026d3a49d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1937,7 +1937,7 @@
         <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Repair target</x:v>

</xml_diff>

<commit_message>
Tighten routed descent repair audit
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rd0f82e026d3a49d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R760dc527b8834829"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1937,7 +1937,7 @@
         <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Repair target</x:v>

</xml_diff>

<commit_message>
Prove normalized law domination dichotomy
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R760dc527b8834829"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R3d8367a614874c79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -911,1587 +911,1604 @@
     </x:row>
     <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law dichotomy</x:v>
       </x:c>
       <x:c r="B40" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Show normalized-law obstruction is forced by failure of finite-rack domination.</x:v>
       </x:c>
       <x:c r="C40" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_domination_dichotomy.md proves finite-rack domination is equivalent to one finite group-longitude detector and that failure diagonalizes to a normalized-law sequence; local residual version included.</x:v>
       </x:c>
       <x:c r="D40" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E40" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>Still need a positive uniform endpoint/descent theorem or an explicit interval with no finite group detector.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E41" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D43" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D44" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D46" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D47" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D55" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D72" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D74" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D113" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D125" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D126" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D127" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D128" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D131" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="48" customHeight="1">
       <x:c r="A132" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="48" customHeight="1">
+      <x:c r="A133" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B132" t="str">
+      <x:c r="B133" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C132" t="str">
+      <x:c r="C133" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D132" t="str">
+      <x:c r="D133" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E132" t="str">
+      <x:c r="E133" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D132">
+  <x:conditionalFormatting sqref="D2:D133">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add normalized law counterexample certificate
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R3d8367a614874c79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R84b78eedc0cc411d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -928,1587 +928,1604 @@
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law B certificate</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E41" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D44" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D45" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D47" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D48" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D56" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D114" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D125" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D126" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D127" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D128" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D129" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D130" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="48" customHeight="1">
       <x:c r="A132" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B132" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D132" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="48" customHeight="1">
       <x:c r="A133" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="48" customHeight="1">
+      <x:c r="A134" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B133" t="str">
+      <x:c r="B134" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C133" t="str">
+      <x:c r="C134" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D133" t="str">
+      <x:c r="D134" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E133" t="str">
+      <x:c r="E134" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D133">
+  <x:conditionalFormatting sqref="D2:D134">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Prove global local normalized fork
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R84b78eedc0cc411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R1f20defcc998405b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -928,1604 +928,1621 @@
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" t="str">
-        <x:v>Normalized-law B certificate</x:v>
+        <x:v>Global-local normalized fork</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
+        <x:v>Remove global ambiguity by reducing Sawin to the local-minimal detector theorem.</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
+        <x:v>proofs/global_local_normalized_fork.md proves maximal chain intervals are local-minimal, local detectors descend to a global finite rack, and local detector failure diagonalizes to a normalized-law residual obstruction; local_normalized_law_prefix_witness_audit checks one supplied local prefix.</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>Certificate format</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E41" t="str">
-        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
+        <x:v>The only remaining theorem is fixed finite detection for each local-minimal interval, especially the bi-free universal-corridor branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law B certificate</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D45" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D46" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D48" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D49" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D74" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D115" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D126" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D127" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D128" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D129" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D130" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D131" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="48" customHeight="1">
       <x:c r="A132" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B132" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="48" customHeight="1">
       <x:c r="A133" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B133" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D133" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="48" customHeight="1">
       <x:c r="A134" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="48" customHeight="1">
+      <x:c r="A135" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B134" t="str">
+      <x:c r="B135" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C134" t="str">
+      <x:c r="C135" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D134" t="str">
+      <x:c r="D135" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E134" t="str">
+      <x:c r="E135" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D134">
+  <x:conditionalFormatting sqref="D2:D135">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Reduce finite detectors to symmetric groups
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R1f20defcc998405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rba0ff5d1096643a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -945,1604 +945,1621 @@
     </x:row>
     <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" t="str">
-        <x:v>Normalized-law B certificate</x:v>
+        <x:v>Symmetric detector reduction</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
+        <x:v>Replace arbitrary finite group detectors by symmetric group detectors.</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
+        <x:v>proofs/symmetric_detector_reduction.md uses the left regular embedding G -&gt; S_m; symmetric_detector_reduction_audit records that K_{S_m} is contained in K_G.</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Certificate format</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
+        <x:v>Positive route may construct S_m detectors; B route may diagonalize against S_j.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law B certificate</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D46" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D47" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D49" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D50" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D58" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D127" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D128" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D129" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D130" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D131" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="48" customHeight="1">
       <x:c r="A132" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B132" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D132" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="48" customHeight="1">
       <x:c r="A133" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B133" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="48" customHeight="1">
       <x:c r="A134" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B134" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D134" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="48" customHeight="1">
       <x:c r="A135" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="48" customHeight="1">
+      <x:c r="A136" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B135" t="str">
+      <x:c r="B136" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C135" t="str">
+      <x:c r="C136" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D135" t="str">
+      <x:c r="D136" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E135" t="str">
+      <x:c r="E136" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D135">
+  <x:conditionalFormatting sqref="D2:D136">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add symmetric tower counterexample certificate
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rba0ff5d1096643a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rf9bff722ba114e0f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -962,1604 +962,1621 @@
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" t="str">
-        <x:v>Normalized-law B certificate</x:v>
+        <x:v>Symmetric-tower B certificate</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
+        <x:v>State the simplified constructive B data after reducing to symmetric groups.</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
+        <x:v>proofs/symmetric_tower_counterexample_certificate.md states that witnesses invisible to S_j for every j suffice; symmetric_normalized_law_prefix_witness_audit and local_symmetric_normalized_law_prefix_witness_audit check supplied rows.</x:v>
       </x:c>
       <x:c r="D43" t="str">
         <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
+        <x:v>A final B proof must still construct the all-j sequence and moved tuples symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law B certificate</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D47" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D48" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D50" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D51" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D121" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D123" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D125" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D126" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D128" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D129" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D130" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D131" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="48" customHeight="1">
       <x:c r="A132" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B132" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D132" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="48" customHeight="1">
       <x:c r="A133" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B133" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D133" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="48" customHeight="1">
       <x:c r="A134" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B134" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="48" customHeight="1">
       <x:c r="A135" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B135" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D135" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="48" customHeight="1">
       <x:c r="A136" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="48" customHeight="1">
+      <x:c r="A137" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B136" t="str">
+      <x:c r="B137" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C136" t="str">
+      <x:c r="C137" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D136" t="str">
+      <x:c r="D137" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E136" t="str">
+      <x:c r="E137" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D136">
+  <x:conditionalFormatting sqref="D2:D137">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add symmetric tower monotonicity
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Rf9bff722ba114e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R75ef0bbe04124096"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -962,1621 +962,1638 @@
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" t="str">
-        <x:v>Symmetric-tower B certificate</x:v>
+        <x:v>Symmetric tower monotonicity</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>State the simplified constructive B data after reducing to symmetric groups.</x:v>
+        <x:v>Record K_{S_M} subset K_{S_m} for M &gt;= m.</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>proofs/symmetric_tower_counterexample_certificate.md states that witnesses invisible to S_j for every j suffice; symmetric_normalized_law_prefix_witness_audit and local_symmetric_normalized_law_prefix_witness_audit check supplied rows.</x:v>
+        <x:v>proofs/symmetric_tower_monotonicity.md proves the fixed-point inclusion argument; symmetric_tower_monotonicity_audit checks supplied braid signatures.</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Certificate format</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>A final B proof must still construct the all-j sequence and moved tuples symbolically.</x:v>
+        <x:v>Positive detector degrees are upward closed; B invisibility to S_j implies eventual invisibility to every fixed S_m.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" t="str">
-        <x:v>Normalized-law B certificate</x:v>
+        <x:v>Symmetric-tower B certificate</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
+        <x:v>State the simplified constructive B data after reducing to symmetric groups.</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
+        <x:v>proofs/symmetric_tower_counterexample_certificate.md states that witnesses invisible to S_j for every j suffice; symmetric_normalized_law_prefix_witness_audit and local_symmetric_normalized_law_prefix_witness_audit check supplied rows.</x:v>
       </x:c>
       <x:c r="D44" t="str">
         <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
+        <x:v>A final B proof must still construct the all-j sequence and moved tuples symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law B certificate</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D48" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D49" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D50" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D51" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D52" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D53" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D60" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D118" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D122" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D125" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D126" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D127" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D129" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D130" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D131" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="48" customHeight="1">
       <x:c r="A132" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B132" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D132" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="48" customHeight="1">
       <x:c r="A133" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B133" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D133" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="48" customHeight="1">
       <x:c r="A134" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B134" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D134" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="48" customHeight="1">
       <x:c r="A135" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B135" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="48" customHeight="1">
       <x:c r="A136" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B136" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D136" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="48" customHeight="1">
       <x:c r="A137" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="48" customHeight="1">
+      <x:c r="A138" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B137" t="str">
+      <x:c r="B138" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C137" t="str">
+      <x:c r="C138" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D137" t="str">
+      <x:c r="D138" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E137" t="str">
+      <x:c r="E138" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D137">
+  <x:conditionalFormatting sqref="D2:D138">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Add local symmetric detector dichotomy
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R75ef0bbe04124096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Raaacaf73d3974a3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -979,1621 +979,1638 @@
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" t="str">
-        <x:v>Symmetric-tower B certificate</x:v>
+        <x:v>Local symmetric detector dichotomy</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>State the simplified constructive B data after reducing to symmetric groups.</x:v>
+        <x:v>Package the final local A/B fork into fixed S_m detection versus S_j movers for every j.</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>proofs/symmetric_tower_counterexample_certificate.md states that witnesses invisible to S_j for every j suffice; symmetric_normalized_law_prefix_witness_audit and local_symmetric_normalized_law_prefix_witness_audit check supplied rows.</x:v>
+        <x:v>proofs/local_symmetric_detector_dichotomy.md proves the dichotomy; local_symmetric_tower_prefix_sequence_audit checks finite supplied prefixes.</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>Certificate format</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>A final B proof must still construct the all-j sequence and moved tuples symbolically.</x:v>
+        <x:v>Still need either a uniform proof of some m(pi,Q), or a symbolic all-j construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Normalized-law B certificate</x:v>
+        <x:v>Symmetric-tower B certificate</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
+        <x:v>State the simplified constructive B data after reducing to symmetric groups.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
+        <x:v>proofs/symmetric_tower_counterexample_certificate.md states that witnesses invisible to S_j for every j suffice; symmetric_normalized_law_prefix_witness_audit and local_symmetric_normalized_law_prefix_witness_audit check supplied rows.</x:v>
       </x:c>
       <x:c r="D45" t="str">
         <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
+        <x:v>A final B proof must still construct the all-j sequence and moved tuples symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law B certificate</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D49" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D50" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D51" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D52" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D53" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D54" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D61" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D62" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D119" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D120" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Product subgroup</x:v>
+        <x:v>Product witnesses</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
+        <x:v>Avoid false common-assignment shortcut.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Subgroup audit implemented for product labels.</x:v>
+        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
+        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
       <x:c r="A123" t="str">
-        <x:v>Product primitivity</x:v>
+        <x:v>Product subgroup</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
+        <x:v>Closed labels lie in subgroup generated by longitude values.</x:v>
       </x:c>
       <x:c r="C123" t="str">
-        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
+        <x:v>Subgroup audit implemented for product labels.</x:v>
       </x:c>
       <x:c r="D123" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E123" t="str">
-        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
+        <x:v>Prove subgroup membership for all product intervals or find failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="48" customHeight="1">
       <x:c r="A124" t="str">
-        <x:v>Product holonomy normalization</x:v>
+        <x:v>Product primitivity</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
+        <x:v>Certify product local-minimality via pair closures in the label groupoid.</x:v>
       </x:c>
       <x:c r="C124" t="str">
-        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
+        <x:v>Swapped/direct label pair-closure helpers added; no partition enumeration required.</x:v>
       </x:c>
       <x:c r="D124" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E124" t="str">
-        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
+        <x:v>Use before applying product holonomy or closed-label B route.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="48" customHeight="1">
       <x:c r="A125" t="str">
-        <x:v>Product holonomy subgroup scan</x:v>
+        <x:v>Product holonomy normalization</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
+        <x:v>Gauge-normalize product label words to the actual finite holonomy group.</x:v>
       </x:c>
       <x:c r="C125" t="str">
-        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
+        <x:v>Helpers and subgroup audit added; coboundary is identity, pairwise branch is C_m-detected, and certificate groups are exposed.</x:v>
       </x:c>
       <x:c r="D125" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
+        <x:v>Prove all-n longitude-subgroup membership in normalized product holonomy groups.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="48" customHeight="1">
       <x:c r="A126" t="str">
-        <x:v>Product holonomy exact scan</x:v>
+        <x:v>Product holonomy subgroup scan</x:v>
       </x:c>
       <x:c r="B126" t="str">
-        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
+        <x:v>Check normalized holonomy subgroup convention in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C126" t="str">
-        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
+        <x:v>Two-colour/two-point fibres: 92 product branch scans; 2048 nonidentity normalized holonomy rows; 0 subgroup failures.</x:v>
       </x:c>
       <x:c r="D126" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
+        <x:v>Search beyond fibre size 2/colour size 2 or prove normalized product holonomy theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="48" customHeight="1">
       <x:c r="A127" t="str">
-        <x:v>Product subgroup scan</x:v>
+        <x:v>Product holonomy exact scan</x:v>
       </x:c>
       <x:c r="B127" t="str">
-        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
+        <x:v>Close fixed-degree normalized holonomy images without word-length cutoff on representative rows.</x:v>
       </x:c>
       <x:c r="C127" t="str">
-        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
+        <x:v>5 exact scenarios; 0 truncations; raw holonomy misses 1 known-branch row; adding S4 removes that miss.</x:v>
       </x:c>
       <x:c r="D127" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E127" t="str">
-        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
+        <x:v>Use full detector product, not raw holonomy alone, in product theorem or B search.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="48" customHeight="1">
       <x:c r="A128" t="str">
-        <x:v>Closed-label B route</x:v>
+        <x:v>Product subgroup scan</x:v>
       </x:c>
       <x:c r="B128" t="str">
-        <x:v>Diagonalize failure of every closed-label detector.</x:v>
+        <x:v>Stress subgroup criterion in smallest arbitrary product corpus.</x:v>
       </x:c>
       <x:c r="C128" t="str">
-        <x:v>Obstruction criterion plus bounded helper.</x:v>
+        <x:v>2-colour fibre-2 all-base scan: 0 failures.</x:v>
       </x:c>
       <x:c r="D128" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E128" t="str">
-        <x:v>Use after explicit all-G product failure.</x:v>
+        <x:v>Escalate beyond fibre size 2 or prove symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="48" customHeight="1">
       <x:c r="A129" t="str">
-        <x:v>2-colour fibre-2</x:v>
+        <x:v>Closed-label B route</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Enumerate identity/flip-base local intervals.</x:v>
+        <x:v>Diagonalize failure of every closed-label detector.</x:v>
       </x:c>
       <x:c r="C129" t="str">
-        <x:v>No unknown primitive examples.</x:v>
+        <x:v>Obstruction criterion plus bounded helper.</x:v>
       </x:c>
       <x:c r="D129" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E129" t="str">
-        <x:v>Search larger colour/fibre patterns.</x:v>
+        <x:v>Use after explicit all-G product failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="48" customHeight="1">
       <x:c r="A130" t="str">
-        <x:v>2-colour fibre-2 all bases</x:v>
+        <x:v>2-colour fibre-2</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
+        <x:v>Enumerate identity/flip-base local intervals.</x:v>
       </x:c>
       <x:c r="C130" t="str">
-        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
+        <x:v>No unknown primitive examples.</x:v>
       </x:c>
       <x:c r="D130" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E130" t="str">
-        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
+        <x:v>Search larger colour/fibre patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="48" customHeight="1">
       <x:c r="A131" t="str">
-        <x:v>2-colour fibre-3 product</x:v>
+        <x:v>2-colour fibre-2 all bases</x:v>
       </x:c>
       <x:c r="B131" t="str">
-        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
+        <x:v>Enumerate arbitrary local tables over all 2-point bases.</x:v>
       </x:c>
       <x:c r="C131" t="str">
-        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>120 local-minimal; no untagged universal corridors.</x:v>
       </x:c>
       <x:c r="D131" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E131" t="str">
-        <x:v>Prove product-groupoid theorem.</x:v>
+        <x:v>Escalate fibre size or prove symbolic branch.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="48" customHeight="1">
       <x:c r="A132" t="str">
-        <x:v>3-colour fibre-2 product</x:v>
+        <x:v>2-colour fibre-3 product</x:v>
       </x:c>
       <x:c r="B132" t="str">
-        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
+        <x:v>Enumerate S3 swapped/direct product labels.</x:v>
       </x:c>
       <x:c r="C132" t="str">
-        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
+        <x:v>Swapped 2064/direct 24 primitive; router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D132" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E132" t="str">
-        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
+        <x:v>Prove product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="48" customHeight="1">
       <x:c r="A133" t="str">
-        <x:v>Linear F2</x:v>
+        <x:v>3-colour fibre-2 product</x:v>
       </x:c>
       <x:c r="B133" t="str">
-        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
+        <x:v>Enumerate S2 product labels over all size-3 quotient bases via F2 linear equations.</x:v>
       </x:c>
       <x:c r="C133" t="str">
-        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
+        <x:v>2472 primitive rows; fibre2 affine router sends all to product_finite_g, 0 open product targets.</x:v>
       </x:c>
       <x:c r="D133" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E133" t="str">
-        <x:v>Search higher-rank affine patterns.</x:v>
+        <x:v>Use fibre-size-two affine detector branch; prove arbitrary-fibre product-groupoid theorem.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="48" customHeight="1">
       <x:c r="A134" t="str">
-        <x:v>Affine F2</x:v>
+        <x:v>Linear F2</x:v>
       </x:c>
       <x:c r="B134" t="str">
-        <x:v>Enumerate translated affine maps on F2^2.</x:v>
+        <x:v>Enumerate all linear bijective maps on F2^2.</x:v>
       </x:c>
       <x:c r="C134" t="str">
-        <x:v>481 YBE; depth1 universals all involutive.</x:v>
+        <x:v>97 YBE tables; no unknown primitive examples; 0 two-strand Sym-gate failures.</x:v>
       </x:c>
       <x:c r="D134" t="str">
         <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>Search non-affine or higher-rank affine.</x:v>
+        <x:v>Search higher-rank affine patterns.</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="48" customHeight="1">
       <x:c r="A135" t="str">
-        <x:v>Known branches</x:v>
+        <x:v>Affine F2</x:v>
       </x:c>
       <x:c r="B135" t="str">
-        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
+        <x:v>Enumerate translated affine maps on F2^2.</x:v>
       </x:c>
       <x:c r="C135" t="str">
-        <x:v>Branch list recorded in proof log.</x:v>
+        <x:v>481 YBE; depth1 universals all involutive.</x:v>
       </x:c>
       <x:c r="D135" t="str">
-        <x:v>Bookkept</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>Focus on arbitrary fibres/colours.</x:v>
+        <x:v>Search non-affine or higher-rank affine.</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="48" customHeight="1">
       <x:c r="A136" t="str">
-        <x:v>Master theorem</x:v>
+        <x:v>Known branches</x:v>
       </x:c>
       <x:c r="B136" t="str">
-        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
+        <x:v>Do not re-open eliminated cases as final obstacles.</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
+        <x:v>Branch list recorded in proof log.</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>Open</x:v>
+        <x:v>Bookkept</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>Prove detection or realize escape.</x:v>
+        <x:v>Focus on arbitrary fibres/colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="48" customHeight="1">
       <x:c r="A137" t="str">
-        <x:v>Counterexample path</x:v>
+        <x:v>Master theorem</x:v>
       </x:c>
       <x:c r="B137" t="str">
-        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+        <x:v>Find uniform G(pi,Q) for local-minimal interval.</x:v>
       </x:c>
       <x:c r="C137" t="str">
-        <x:v>No candidate yet.</x:v>
+        <x:v>Kernel/Schutzenberger group candidate isolated.</x:v>
       </x:c>
       <x:c r="D137" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E137" t="str">
-        <x:v>Search for normalized-law behavior.</x:v>
+        <x:v>Prove detection or realize escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="48" customHeight="1">
       <x:c r="A138" t="str">
+        <x:v>Counterexample path</x:v>
+      </x:c>
+      <x:c r="B138" t="str">
+        <x:v>Explicit X, symbolic YBE, beta_j, moved tuple.</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>No candidate yet.</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>Search for normalized-law behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="48" customHeight="1">
+      <x:c r="A139" t="str">
         <x:v>GPT-5.5 Pro audit</x:v>
       </x:c>
-      <x:c r="B138" t="str">
+      <x:c r="B139" t="str">
         <x:v>Ask critic before finalizing A or B.</x:v>
       </x:c>
-      <x:c r="C138" t="str">
+      <x:c r="C139" t="str">
         <x:v>Awaiting final candidate.</x:v>
       </x:c>
-      <x:c r="D138" t="str">
+      <x:c r="D139" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="E138" t="str">
+      <x:c r="E139" t="str">
         <x:v>Use Browser/Chrome for final audit.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="D2:D138">
+  <x:conditionalFormatting sqref="D2:D139">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Executable"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Conditional"/>

</xml_diff>

<commit_message>
Bridge repair contract to symmetric detectors
</commit_message>
<xml_diff>
--- a/tables/reduction_audit.xlsx
+++ b/tables/reduction_audit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="Raaacaf73d3974a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reduction Audit" sheetId="1" r:id="R9ed1af4fcfaa447a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -996,1621 +996,1638 @@
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" t="str">
-        <x:v>Symmetric-tower B certificate</x:v>
+        <x:v>Symmetric repair bridge</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>State the simplified constructive B data after reducing to symmetric groups.</x:v>
+        <x:v>Translate a successful repair-contract product detector H(pi,Q) into one symmetric detector degree.</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>proofs/symmetric_tower_counterexample_certificate.md states that witnesses invisible to S_j for every j suffice; symmetric_normalized_law_prefix_witness_audit and local_symmetric_normalized_law_prefix_witness_audit check supplied rows.</x:v>
+        <x:v>proofs/symmetric_repair_contract_bridge.md proves that if the supplied repair contract gives H, then S_m with m&gt;=|H| also detects; symmetric_repair_contract_bridge_audit records the bridge.</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Certificate format</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>A final B proof must still construct the all-j sequence and moved tuples symbolically.</x:v>
+        <x:v>Still need the repair contract's fixed descent readout, faithful decomposition, and all-n endpoint witnesses.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" t="str">
-        <x:v>Normalized-law B certificate</x:v>
+        <x:v>Symmetric-tower B certificate</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
+        <x:v>State the simplified constructive B data after reducing to symmetric groups.</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
+        <x:v>proofs/symmetric_tower_counterexample_certificate.md states that witnesses invisible to S_j for every j suffice; symmetric_normalized_law_prefix_witness_audit and local_symmetric_normalized_law_prefix_witness_audit check supplied rows.</x:v>
       </x:c>
       <x:c r="D46" t="str">
         <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
+        <x:v>A final B proof must still construct the all-j sequence and moved tuples symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" t="str">
-        <x:v>Small YBE scan</x:v>
+        <x:v>Normalized-law B certificate</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
+        <x:v>Separate constructive B data from nonconstructive all-detector failure.</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>Size-2 full, size-3 capped scan.</x:v>
+        <x:v>proofs/normalized_law_counterexample_certificate.md states the product-prefix witness format; normalized_law_prefix_witness_audit checks one supplied prefix for product invisibility, right stabilization, and moved tuples.</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Certificate format</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>Escalate beyond tiny tables.</x:v>
+        <x:v>A final B proof must supply these prefix witnesses for every product P_j, not just a bounded detector miss.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" t="str">
-        <x:v>Size-3 candidates</x:v>
+        <x:v>Small YBE scan</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
+        <x:v>Screen tiny YBE tables for law-braid motion.</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>Report generated; affine and S3-visible.</x:v>
+        <x:v>Size-2 full, size-3 capped scan.</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>Candidate only</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>Need all-finite-group law sequence.</x:v>
+        <x:v>Escalate beyond tiny tables.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" t="str">
-        <x:v>Green branch</x:v>
+        <x:v>Size-3 candidates</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>Audit coordinate-action monoid branch choices.</x:v>
+        <x:v>Detail nonrack tables moved by commutator law braid.</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
+        <x:v>Report generated; affine and S3-visible.</x:v>
       </x:c>
       <x:c r="D49" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate only</x:v>
       </x:c>
       <x:c r="E49" t="str">
-        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
+        <x:v>Need all-finite-group law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" t="str">
-        <x:v>Local-minimal Green</x:v>
+        <x:v>Green branch</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>Run Green loops through congruence-cover intervals.</x:v>
+        <x:v>Audit coordinate-action monoid branch choices.</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>Universal-output Green overlaps all known.</x:v>
+        <x:v>Atom descent closure, descent-closed rack quotient, atom inner group, and unit-lift detector criterion recorded; two-sided Green detector list now includes atom inner groups.</x:v>
       </x:c>
       <x:c r="D50" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>Prove all-n finite-G detection.</x:v>
+        <x:v>Prove descent closure is trivial/absorbed and endpoint-unit subgroup membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" t="str">
-        <x:v>Kernel detectors</x:v>
+        <x:v>Local-minimal Green</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>Compare kernel image vs Sym blocks.</x:v>
+        <x:v>Run Green loops through congruence-cover intervals.</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
+        <x:v>Universal-output Green overlaps all known.</x:v>
       </x:c>
       <x:c r="D51" t="str">
         <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E51" t="str">
-        <x:v>Prove symmetric kernel groups suffice.</x:v>
+        <x:v>Prove all-n finite-G detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" t="str">
-        <x:v>Dual Green</x:v>
+        <x:v>Kernel detectors</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>Include right-coordinate Green kernel data.</x:v>
+        <x:v>Compare kernel image vs Sym blocks.</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
+        <x:v>No len&lt;=4 collisions; exact n=2 closes.</x:v>
       </x:c>
       <x:c r="D52" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E52" t="str">
-        <x:v>Prove two-sided Green detection.</x:v>
+        <x:v>Prove symmetric kernel groups suffice.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" t="str">
-        <x:v>Opposite detectability</x:v>
+        <x:v>Dual Green</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
+        <x:v>Include right-coordinate Green kernel data.</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
+        <x:v>Opposite audit plus two-sided Sym helper.</x:v>
       </x:c>
       <x:c r="D53" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E53" t="str">
-        <x:v>Use same detector factors on left/right dual branches.</x:v>
+        <x:v>Prove two-sided Green detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" t="str">
-        <x:v>Semigroup holonomy</x:v>
+        <x:v>Opposite detectability</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
+        <x:v>Finite-G detectability is invariant under side-opposite solution.</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
+        <x:v>Strand-reversal proof plus braid-action and longitude invariance tests.</x:v>
       </x:c>
       <x:c r="D54" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
+        <x:v>Use same detector factors on left/right dual branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" t="str">
-        <x:v>Green holonomy gate</x:v>
+        <x:v>Semigroup holonomy</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
+        <x:v>Separate group holonomy from aperiodic reset parts.</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
+        <x:v>Aperiodic lemma, endpoint/product expression audits with explicit product witnesses, product-unit detector, and endpoint finite-failure flags recorded.</x:v>
       </x:c>
       <x:c r="D55" t="str">
-        <x:v>Executable guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E55" t="str">
-        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
+        <x:v>Display all-n residual endpoint units as longitude expressions in a fixed unit group, or prove subgroup membership directly.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" t="str">
-        <x:v>Involutive/permutation</x:v>
+        <x:v>Green holonomy gate</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>Known branch finite-rack domination.</x:v>
+        <x:v>Separate raw atom-trivial context collapse from group-like completed-context holonomy.</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
+        <x:v>Loop unit groups extracted; endpoint-product flags record direct membership in one detector.</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>Symbolic branch proof</x:v>
+        <x:v>Executable guardrail</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>Use as closed branch in local bottleneck routing.</x:v>
+        <x:v>Prove these group-like loops factor through fixed H(pi,Q), or build B in this group part.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" t="str">
-        <x:v>Affine tag guardrail</x:v>
+        <x:v>Involutive/permutation</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
+        <x:v>Known branch finite-rack domination.</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
+        <x:v>T2 for involutive; C_m twist detector plus pure-longitude tests; known_branch_detector_certificate exposes G and |A_G|.</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>Proof hygiene</x:v>
+        <x:v>Symbolic branch proof</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
+        <x:v>Use as closed branch in local bottleneck routing.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" t="str">
-        <x:v>Structure orbits</x:v>
+        <x:v>Affine tag guardrail</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>Separate product invariants from orbit holonomy.</x:v>
+        <x:v>Prevent audit-only affine_cyclic tags from closing a local interval.</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>Orbit factors plus correlated global image profiled.</x:v>
+        <x:v>Regression excludes affine_cyclic from KNOWN_TOTAL_DETECTOR_TAGS; proof note added.</x:v>
       </x:c>
       <x:c r="D58" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof hygiene</x:v>
       </x:c>
       <x:c r="E58" t="str">
-        <x:v>Detect holonomy in correlated global image.</x:v>
+        <x:v>Use affine rows only via a symbolic all-n detector branch or a closed product subbranch.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" t="str">
-        <x:v>Bounded-degree images</x:v>
+        <x:v>Structure orbits</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
+        <x:v>Separate product invariants from orbit holonomy.</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
+        <x:v>Orbit factors plus correlated global image profiled.</x:v>
       </x:c>
       <x:c r="D59" t="str">
-        <x:v>Guardrail</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
+        <x:v>Detect holonomy in correlated global image.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" t="str">
-        <x:v>Orbit-law obstruction</x:v>
+        <x:v>Bounded-degree images</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
+        <x:v>Do not use rho_X(B_n) or orbit groups as n-dependent detectors.</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
+        <x:v>proofs/bounded_degree_action_image_limit.md records the limitation.</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>Proof criterion</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
+        <x:v>Replace fixed-degree images by an all-n factorization through fixed G.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" t="str">
-        <x:v>Context retraction</x:v>
+        <x:v>Orbit-law obstruction</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>Two-sided context-profile congruence.</x:v>
+        <x:v>Localize normalized-law B route to one structure orbit.</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
+        <x:v>Assigned-generator helper; Sym-law audit has 0 tiny failures.</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Proof criterion</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Prove two-sided-free branch detection.</x:v>
+        <x:v>Upgrade orbit-local separators to all-j sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" t="str">
-        <x:v>Coretraction</x:v>
+        <x:v>Context retraction</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>Dual two-sided input-profile congruence.</x:v>
+        <x:v>Two-sided context-profile congruence.</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
+        <x:v>Symbolic admissible; size&lt;=3 split.</x:v>
       </x:c>
       <x:c r="D62" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E62" t="str">
-        <x:v>Prove bi-free branch detection.</x:v>
+        <x:v>Prove two-sided-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" t="str">
-        <x:v>Bi-free rank</x:v>
+        <x:v>Coretraction</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>Rank/kernel profile for bi-free rows.</x:v>
+        <x:v>Dual two-sided input-profile congruence.</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>No untagged size3 rank/kernel rows.</x:v>
+        <x:v>Symbolic admissible; bi-free size3 known.</x:v>
       </x:c>
       <x:c r="D63" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E63" t="str">
-        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
+        <x:v>Prove bi-free branch detection.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" t="str">
-        <x:v>Local bottleneck</x:v>
+        <x:v>Bi-free rank</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>Route each local interval to a branch verdict.</x:v>
+        <x:v>Rank/kernel profile for bi-free rows.</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
+        <x:v>No untagged size3 rank/kernel rows.</x:v>
       </x:c>
       <x:c r="D64" t="str">
-        <x:v>Reduction ledger</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
+        <x:v>Prove rank/Green dichotomy symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" t="str">
-        <x:v>Bi-free corridor target</x:v>
+        <x:v>Local bottleneck</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
+        <x:v>Route each local interval to a branch verdict.</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
+        <x:v>Router records explicit known/product detectors, one product group per closed row, and closed_detector_gaps for delegated/open rows.</x:v>
       </x:c>
       <x:c r="D65" t="str">
-        <x:v>Open theorem target</x:v>
+        <x:v>Reduction ledger</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
+        <x:v>Prove genuinely-coloured product or bi-free corridor factorization, or realize B there.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" t="str">
-        <x:v>Bi-free endpoint factorization</x:v>
+        <x:v>Bi-free corridor target</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
+        <x:v>State exact hypotheses, fixed H(pi,Q), and B certificate.</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
+        <x:v>Target note added; false rack/Hurwitz shortcuts excluded; corridor helpers now accept fixed extra detector factors for quotient/known/unit components of H(pi,Q).</x:v>
       </x:c>
       <x:c r="D66" t="str">
-        <x:v>Assembly lemma</x:v>
+        <x:v>Open theorem target</x:v>
       </x:c>
       <x:c r="E66" t="str">
-        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
+        <x:v>Prove all-n H(pi,Q) factorization or build normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" t="str">
-        <x:v>Artin-defect sieve</x:v>
+        <x:v>Bi-free endpoint factorization</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
+        <x:v>Assemble corridor endpoint-longitude expressions into one fixed product detector.</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
+        <x:v>Endpoint expression/readout/action helpers build product witnesses, verify faithful rows, and separate supplied-row proof from row-coverage claims; the Artin-defect sieve now converts displayed beta(w)p(w)^-1 endpoint values into longitude-subgroup witnesses.</x:v>
       </x:c>
       <x:c r="D67" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Assembly lemma</x:v>
       </x:c>
       <x:c r="E67" t="str">
-        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
+        <x:v>Prove the sharpened Artin-defect endpoint lemma for every target interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" t="str">
-        <x:v>Artin detector lift</x:v>
+        <x:v>Artin-defect sieve</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
+        <x:v>Replace arbitrary endpoint-longitude search by Artin permutation defect displays.</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
+        <x:v>proofs/artin_defect_longitudinalization_sieve.md proves defects beta(w)p_beta(w)^-1 lie in the normal closure of recursive longitudes; endpoint_artin_defect_audit and endpoint_product_artin_defect_audit verify supplied displays.</x:v>
       </x:c>
       <x:c r="D68" t="str">
-        <x:v>Finite row criterion</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E68" t="str">
-        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
+        <x:v>Display every elementary Green/corridor endpoint generator as a finite product of Artin-defect values in fixed H(pi,Q) factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" t="str">
-        <x:v>Atom-inner row lift</x:v>
+        <x:v>Artin detector lift</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
+        <x:v>Turn endpoint observers with live (m,u) labels into recursive longitude expressions.</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
+        <x:v>proofs/artin_detector_lift_criterion.md proves the unbounded braid recursion from finite U x U row identities; artin_detector_lift_transition_audit and artin_detector_lift_braid_audit verify rows and convention.</x:v>
       </x:c>
       <x:c r="D69" t="str">
-        <x:v>Conditional closure</x:v>
+        <x:v>Finite row criterion</x:v>
       </x:c>
       <x:c r="E69" t="str">
-        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
+        <x:v>Verify the detector-lift identities for every remaining Green/corridor observer row in fixed factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" t="str">
-        <x:v>Green first-output defect</x:v>
+        <x:v>Atom-inner row lift</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
+        <x:v>Close the rack-like atom quotient inner-group detector-lift rows.</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
+        <x:v>proofs/atom_inner_detector_lift_rows.md proves positive rows from L_{a*b}=L_a L_b L_a^-1 and negative rows as inverse positive rows; rack_inner_detector_lift_audit and atom_quotient_inner_detector_lift_audit expose the check.</x:v>
       </x:c>
       <x:c r="D70" t="str">
-        <x:v>Sharper open target</x:v>
+        <x:v>Conditional closure</x:v>
       </x:c>
       <x:c r="E70" t="str">
-        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
+        <x:v>Still prove atom descent/totality; remaining row checks are Green kernel-block, Schutzenberger, and endpoint/unit holonomy factors.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" t="str">
-        <x:v>Green defect quotient</x:v>
+        <x:v>Green first-output defect</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
+        <x:v>Replace Green kernel-block/Schutzenberger row checks by one transported defect endpoint.</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
+        <x:v>proofs/green_first_output_defect_criterion.md proves the row normal form from g(a)g(q)=g(q^a)g(a^q); schutzenberger_kernel_defect_pushforward_audits checks kernel pushforwards.</x:v>
       </x:c>
       <x:c r="D71" t="str">
-        <x:v>Quotient closure</x:v>
+        <x:v>Sharper open target</x:v>
       </x:c>
       <x:c r="E71" t="str">
-        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
+        <x:v>Pass to the defect-kernel quotient, then handle local-only and lower endpoint/unit holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" t="str">
-        <x:v>Green defect potential</x:v>
+        <x:v>Green defect quotient</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
+        <x:v>Kill all non-defect Green/Schutzenberger row motion by a fixed quotient.</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
+        <x:v>proofs/green_defect_kernel_quotient_detection.md quotients each observer U_C by the normal closure Def_C of its first-output defects; projected rows are exact side-opposite rack-Artin and green_defect_kernel_quotient_audit verifies the finite quotient step.</x:v>
       </x:c>
       <x:c r="D72" t="str">
-        <x:v>Coboundary reduction</x:v>
+        <x:v>Quotient closure</x:v>
       </x:c>
       <x:c r="E72" t="str">
-        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
+        <x:v>Prove the remaining defect-kernel endpoint D_C(beta) lies in V_beta(Def_C), preferably by Artin-defect displays.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" t="str">
-        <x:v>Artin-defect abelianization</x:v>
+        <x:v>Green defect potential</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
+        <x:v>Reduce elementary Def_C defects to a finite nonabelian coboundary on retained edge-germs.</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
+        <x:v>proofs/green_defect_potential_coboundary.md proves d(a,q)=eta(q^a)eta(q)^-1 after choosing a base edge per defect component; green_defect_kernel_potential_audit verifies potentials lie in Def_C and all row coboundaries match.</x:v>
       </x:c>
       <x:c r="D73" t="str">
-        <x:v>Proof guardrail</x:v>
+        <x:v>Coboundary reduction</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
+        <x:v>Prove the Def_C potential is principal for Artin detector transport, or extract a normalized-law cocycle escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" t="str">
-        <x:v>Green defect abelian split</x:v>
+        <x:v>Artin-defect abelianization</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
+        <x:v>Prevent an invalid elementary Artin-defect display proof for abelian defect kernels.</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
+        <x:v>proofs/artin_defect_abelianization_barrier.md proves Artin permutation defects land in [K,K]; the affine Green stress row has Def_C=C3 and nonidentity row defects outside [Def_C,Def_C].</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Proof guardrail</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
+        <x:v>Use full recursive-longitude membership, endpoint cancellation, or detector-lift labels for abelian defect-kernel data.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" t="str">
-        <x:v>Abelian longitude image</x:v>
+        <x:v>Green defect abelian split</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
+        <x:v>Separate the finite abelian defect quotient from the commutator endpoint.</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
+        <x:v>proofs/green_defect_abelianization_split.md records the split Def_C -&gt; Def_C/[Def_C,Def_C]; green_defect_abelianization_split_audit verifies the projected potential coboundaries.</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Exact criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
+        <x:v>Prove ordinary finite abelian longitude visibility for the projected endpoint, then handle the commutator residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" t="str">
-        <x:v>Green balanced gauge</x:v>
+        <x:v>Abelian longitude image</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
+        <x:v>Compute V_beta(A) exactly for any fixed finite abelian target.</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
+        <x:v>proofs/abelian_longitude_image_criterion.md proves V_beta(A)=&lt;a^{m_ij}&gt; from the recursive-longitude exponent matrix; abelian_longitude_image_audit optionally checks the matrix subgroup against exhaustive enumeration.</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Exact criterion</x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
+        <x:v>Apply this matrix subgroup to the projected AbDef_C endpoint, then route the remaining commutator endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" t="str">
-        <x:v>Terminal gauge criterion</x:v>
+        <x:v>Green balanced gauge</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
+        <x:v>Split raw Green/Schutzenberger first-output defects into Artin-visible commutators plus terminal gauge.</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
+        <x:v>proofs/green_balanced_defect_gauge_decomposition.md proves d=[A,Q]*Q(CA^-1)^-1Q^-1; row audits now expose second_output_gauge and balanced_decomposition_holds.</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Certificate criterion</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
+        <x:v>Prove terminal gauge holonomy lies in the fixed endpoint/unit longitude subgroup.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" t="str">
-        <x:v>Principal gauge extension</x:v>
+        <x:v>Terminal gauge criterion</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
+        <x:v>Turn terminal second-output gauge holonomy into the standard endpoint-longitude certificate target.</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
+        <x:v>proofs/terminal_gauge_longitudinalization_criterion.md proves the gauge telescope and records terminal_gauge_* audits that reuse endpoint expression/product witnesses.</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Closed subcase</x:v>
+        <x:v>Certificate criterion</x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
+        <x:v>Supply all-n terminal gauge certificates in fixed factors, or extract normalized-law gauge escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" t="str">
-        <x:v>Transport-state rackification</x:v>
+        <x:v>Principal gauge extension</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
+        <x:v>Close lower endpoint/unit holonomy when the surviving gauge row is a principal finite rack-extension cocycle.</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
+        <x:v>proofs/principal_gauge_extension_detector.md proves the rack-cocycle criterion; principal_gauge_extension_detector_audit builds A x U and checks Inn(A x U) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
+        <x:v>Prove principal-gauge normal form for every surviving corridor gauge row, or extract a nonprincipal normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" t="str">
-        <x:v>Continuation congruence gate</x:v>
+        <x:v>Transport-state rackification</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
+        <x:v>Remove principality for strand-continuing finite gauge rows by enlarging the rack state to A x E.</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
+        <x:v>proofs/transport_state_rackification_detector.md proves the rackification lemma; transport_state_rackification_audit builds A x E and checks Inn(A x E) detector-lift rows.</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Closed subcase</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
+        <x:v>Prove descent separation: non-strand-continuing motion is fully visible in Green/Schutzenberger readouts.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" t="str">
-        <x:v>Elementary continuation closure</x:v>
+        <x:v>Continuation congruence gate</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
+        <x:v>Turn non-strand-continuing lower motion into a least admissible congruence closure.</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
+        <x:v>proofs/continuation_congruence_descent_gate.md; continuation_congruence_audit seeds x~v and reuses the generated congruence closure engine.</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
+        <x:v>Handle the universal continuation corridor by Green/Schutzenberger visibility, or build a normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" t="str">
-        <x:v>Universal continuation derivation</x:v>
+        <x:v>Elementary continuation closure</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
+        <x:v>Rule out collective-only universal continuation in local-minimal intervals.</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
+        <x:v>proofs/elementary_continuation_closure.md; continuation_seed_pair_closure_audits closes each nontrivial x~v seed separately.</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
+        <x:v>Prove Green/Schutzenberger visibility or normalized-law escape for one representative elementary continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" t="str">
-        <x:v>Continuation readout propagation</x:v>
+        <x:v>Universal continuation derivation</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
+        <x:v>Expose the edge-by-edge finite derivation certificate generated by one universal continuation seed.</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
+        <x:v>proofs/universal_continuation_derivation_certificate.md; continuation_seed_universal_derivation_audits compares edge counts with recorded derivation rows.</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
+        <x:v>Route each derived edge through fixed Green/Schutzenberger/atom readouts, or choose one derived edge as the normalized-law seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" t="str">
-        <x:v>Readout-kernel admissibility</x:v>
+        <x:v>Continuation readout propagation</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
+        <x:v>Show that an admissible fixed readout containing one continuation seed contains the whole generated closure.</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
+        <x:v>proofs/continuation_readout_propagation.md; continuation_seed_readout_propagation_audits records admissibility, seed containment, and missing generated edges.</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
+        <x:v>Prove representative seed visibility in an admissible fixed readout; derived edges then propagate automatically.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" t="str">
-        <x:v>Readout descent separation</x:v>
+        <x:v>Readout-kernel admissibility</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
+        <x:v>Certify when finite fibrewise detector labels define an admissible local congruence kernel.</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
+        <x:v>proofs/readout_kernel_admissibility.md; readout_kernel_audit builds the kernel family and records exact transport failures.</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
+        <x:v>Construct fixed Green/Schutzenberger/atom/unit labels whose kernel is admissible and contains each representative continuation seed.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" t="str">
-        <x:v>Readout quotient interval</x:v>
+        <x:v>Readout descent separation</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
+        <x:v>Combine readout-kernel admissibility and continuation seed killing into a strand-continuing quotient certificate.</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
+        <x:v>proofs/readout_descent_separation_certificate.md; readout_descent_separation_audit records the kernel, propagation audits, and surviving seed rows.</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
+        <x:v>Construct fixed detector labels that make this audit pass in every local-minimal bottleneck interval.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" t="str">
-        <x:v>Product readout kernels</x:v>
+        <x:v>Readout quotient interval</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
+        <x:v>Construct the explicit finite local interval on readout-kernel blocks.</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
+        <x:v>proofs/readout_kernel_quotient_interval.md; quotient_interval_by_family and readout_kernel_quotient_interval build the descended local table.</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
+        <x:v>After a passing descent-separation audit, apply transport-state rackification to the explicit strand-continuing quotient row.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" t="str">
-        <x:v>Product descent separation</x:v>
+        <x:v>Product readout kernels</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
+        <x:v>Assemble finitely many fixed detector labels into one tuple-valued readout.</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
+        <x:v>proofs/product_readout_kernel_assembly.md; product_readout_kernel_audit checks factor kernels, the product kernel, and the meet identity.</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
+        <x:v>Construct Green/Schutzenberger/atom/unit factors separately, then assemble the fixed product readout for descent separation.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" t="str">
-        <x:v>Readout seed saturation</x:v>
+        <x:v>Product descent separation</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
+        <x:v>Track exactly which continuation seeds survive a tuple-valued product readout.</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
+        <x:v>proofs/product_readout_descent_separation.md; product_readout_descent_separation_audit checks factor seed survival and product descent separation.</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
+        <x:v>Each factor must kill every representative continuation seed; one killing factor is not enough because product kernels are meets.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" t="str">
-        <x:v>Local-minimal seed dichotomy</x:v>
+        <x:v>Readout seed saturation</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
+        <x:v>Compute the least admissible coarsening forced by one readout factor plus all continuation seeds.</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
+        <x:v>proofs/readout_seed_saturation.md; readout_seed_saturation_audit records saturation, new edges, and saturated descent separation.</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
+        <x:v>In local-minimal intervals a non-killing admissible equality factor saturates to universal, so lost information must be routed elsewhere.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" t="str">
-        <x:v>Lost-edge external routing</x:v>
+        <x:v>Local-minimal seed dichotomy</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
+        <x:v>Use local-minimality to rule out hidden proper seed-saturated quotients.</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
+        <x:v>proofs/local_minimal_seed_saturation_dichotomy.md; local_minimal_seed_saturation_dichotomy_audit checks the equality/universal saturation expectation.</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
+        <x:v>Any equality-kernel factor missing a nontrivial seed collapses to universal; prove external routing for information lost by that collapse.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" t="str">
-        <x:v>Routed edge endpoint witnesses</x:v>
+        <x:v>Lost-edge external routing</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
+        <x:v>Separate descent quotient labels from external labels that remember collapsed edges.</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
+        <x:v>proofs/lost_edge_external_routing.md; lost_edge_external_routing_audit lists lost, routed, and unrouted saturation edges.</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
+        <x:v>Do not add routing labels back to the descent quotient; prove their fixed-factor longitude visibility separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" t="str">
-        <x:v>Chart-transport collapse</x:v>
+        <x:v>Routed edge endpoint witnesses</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
+        <x:v>Attach product endpoint-longitude certificates to externally routed lost edges.</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
+        <x:v>proofs/routed_lost_edge_endpoint_witness.md; routed_lost_edge_endpoint_witness_audit checks routed-edge coverage by endpoint product-expression audits.</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
+        <x:v>Every routed lost edge still needs a fixed-factor recursive-longitude witness; missing witnesses are not B without normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" t="str">
-        <x:v>Descent separation target</x:v>
+        <x:v>Chart-transport collapse</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
+        <x:v>Avoid separate endpoint-longitude proofs for transported or chart-conjugate copies of elementary generators.</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
+        <x:v>proofs/chart_transport_collapse.md; conjugate_longitude_subgroup_witness shows V_beta(G) is normal at certificate level.</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Closed by final assembly</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
+        <x:v>Prove one representative elementary generator per finite chart-conjugacy orbit.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" t="str">
-        <x:v>Unit-continuation final obstruction</x:v>
+        <x:v>Descent separation target</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
+        <x:v>State the final A-route theorem: all residual endpoint motion separates into fixed Green/Sch, atom, and transport-rack readouts.</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
+        <x:v>proofs/descent_separation_transport_rack_closure.md records the target; later unit-continuation, mixed-unit, triangular, kink-predecessor, and master-local notes route the remaining descent-separation cases.</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>Routed by later closure</x:v>
+        <x:v>Closed by final assembly</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
+        <x:v>Audit the route through proofs/master_local_residual_positive_closure.md and proofs/final_completion_audit.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" t="str">
-        <x:v>Two-sided unit collapse</x:v>
+        <x:v>Unit-continuation final obstruction</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
+        <x:v>Split the constant-observer universal-continuation case into nonunit impossibility and unit endpoint holonomy.</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
+        <x:v>proofs/unit_continuation_final_obstruction.md specializes unit_factorization_audit to Theta^cont=Nabla and K^O=Nabla.</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Routed by later closure</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
+        <x:v>Follow the two-sided unit, mixed-unit, triangular, and kink-predecessor rows to the master-local positive closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" t="str">
-        <x:v>Mixed-unit companion separation</x:v>
+        <x:v>Two-sided unit collapse</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
+        <x:v>Split the final continuation rows into strand-continuing, two-sided unit nondegenerate, and mixed-unit context recovery.</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
+        <x:v>proofs/two_sided_unit_collapse.md; two_sided_unit_collapse_audit records coordinate-section units, non-two-sided rows, and mixed rows.</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
+        <x:v>Mixed-unit rows pass through rank-profile and triangular reductions; two-sided unit and strand-continuing rows are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" t="str">
-        <x:v>Mixed-unit rank-profile collapse</x:v>
+        <x:v>Mixed-unit companion separation</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
+        <x:v>Show every noninjective coordinate-section kernel is separated by the companion output coordinate.</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
+        <x:v>proofs/mixed_unit_companion_separation.md; section_kernel_companion_audit records section collisions and companion outputs.</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Routed by triangular closure</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
+        <x:v>Route companion-shuttle edges through fixed readouts, or upgrade a shuttle cycle to normalized laws.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" t="str">
-        <x:v>Triangular bundle partition</x:v>
+        <x:v>Mixed-unit rank-profile collapse</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
+        <x:v>Route proper section-kernel profiles through Green/Schutzenberger readouts and leave only constant-section triangular rows.</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
+        <x:v>proofs/rank_profile_collapse_mixed_unit.md; section_rank_profile_collapse_audit records ranks, kernel kinds, and images.</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
+        <x:v>Constant-section triangular rows are handled by the triangular bundle, constant-column, Latin split, and kink-predecessor notes.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" t="str">
-        <x:v>Triangular recovery inverse</x:v>
+        <x:v>Triangular bundle partition</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
+        <x:v>Show bijective constant-section triangular rows are finite bundle partitions over the constant output map.</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
+        <x:v>proofs/constant_section_triangular_bundle_partition.md; triangular_bundle_audit records constant-map fibres and companion image blocks.</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
+        <x:v>The recovery inverse and constant-column collapse reduce the bundle residue to Latin-unit triangular rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" t="str">
-        <x:v>Constant-column collapse</x:v>
+        <x:v>Triangular recovery inverse</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
+        <x:v>Compute the inverse of a triangular bundle row from block-label recovery plus within-block companion inverse.</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
+        <x:v>proofs/triangular_bundle_recovery_inverse.md; triangular_recovery_audit records output-to-source recovery entries.</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Reduced to Latin closure</x:v>
+        <x:v>Routed by triangular closure</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
+        <x:v>Constant-column collapse and Latin YBE split remove the non-Latin recovery residue and isolate companion shear.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" t="str">
-        <x:v>Latin triangular YBE split</x:v>
+        <x:v>Constant-column collapse</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
+        <x:v>Show hidden nonunit opposite columns in triangular rows force product/permutation form, leaving only Latin-unit triangular rows.</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
+        <x:v>proofs/constant_column_collapse_triangular.md; triangular_column_collapse_audit records companion sections, opposite columns, product-collapse rows, and Latin-unit rows.</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Routed by kink closure</x:v>
+        <x:v>Reduced to Latin closure</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
+        <x:v>Latin-unit rows are handled by the Latin YBE split, one-colour collapse, and kink-predecessor cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" t="str">
-        <x:v>One-colour Latin triangular collapse</x:v>
+        <x:v>Latin triangular YBE split</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
+        <x:v>Separate alpha transport from companion shear in the Latin-unit triangular residue.</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
+        <x:v>proofs/latin_triangular_ybe_split.md; latin_triangular_ybe_audit records alpha-cocycle, middle-companion, and endpoint-shear YBE equations.</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Colour reduction</x:v>
+        <x:v>Routed by kink closure</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
+        <x:v>Alpha transport routes to product/permutation holonomy; companion shear is eliminated by one-colour and rack-kink cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" t="str">
-        <x:v>Kink-predecessor Latin cancellation</x:v>
+        <x:v>One-colour Latin triangular collapse</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
+        <x:v>Rule out nontrivial one-colour Latin-unit triangular YBE rows.</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
+        <x:v>proofs/one_colour_latin_triangular_collapse.md; one_color_latin_triangular_collapse_audit records alpha identity, companion identity, and rejected Latin shear candidates.</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Local closure input</x:v>
+        <x:v>Colour reduction</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
+        <x:v>Any remaining companion-shear obstruction must be genuinely multi-colour.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" t="str">
-        <x:v>Master local positive closure</x:v>
+        <x:v>Kink-predecessor Latin cancellation</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
+        <x:v>Use rack kink predecessors to prove rack-base Latin-unit triangular rows have singleton fibres.</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
+        <x:v>proofs/kink_predecessor_latin_triangular_cancellation.md; rack_kink_latin_triangular_collapse_audit records rack form, kink predecessors, alpha identities, and predecessor-column constancy.</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Gap found</x:v>
+        <x:v>Local closure input</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
+        <x:v>Feeds the master local positive closure by eliminating the final rack-base Latin-unit triangular obstruction.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" t="str">
-        <x:v>Proof critic gap audit</x:v>
+        <x:v>Master local positive closure</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
+        <x:v>Assemble the fixed detector product H(pi,Q), the bi-free corridor closure, sharp obstruction step, and congruence-chain induction.</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
+        <x:v>proofs/master_local_residual_positive_closure.md is now treated as a candidate assembly template; proofs/proof_critic_gap_audit.md finds that the endpoint expressions, faithful decomposition, and descent separation are not yet proved.</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Current gap</x:v>
+        <x:v>Gap found</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
+        <x:v>Prove uniform descent-separation and endpoint-longitudinalization, or construct normalized-law B.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" t="str">
-        <x:v>Descent-endpoint repair contract</x:v>
+        <x:v>Proof critic gap audit</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
+        <x:v>Record the external proof-critic rejection of the candidate A closure and identify the missing theorem package.</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
+        <x:v>proofs/proof_critic_gap_audit.md states that bifree endpoint factorization is conditional, descent separation remains unproved, atom descent/routing is conditional, and terminal gauge is reduced but not killed.</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Repair target</x:v>
+        <x:v>Current gap</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
+        <x:v>Supply the missing fixed-factor endpoint expressions and faithful residual decomposition uniformly in n.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" t="str">
-        <x:v>Superseded completion audit</x:v>
+        <x:v>Descent-endpoint repair contract</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
+        <x:v>Turn the proof-critic gap into a precise sufficient theorem package.</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
+        <x:v>proofs/descent_endpoint_repair_contract.md proves that a fixed descent-separating readout, fixed endpoint groups, faithful reconstruction, and all-n V_beta witnesses imply the local finite-detector implication; descent_endpoint_repair_contract_audit bundles supplied certificates and rejects mismatched routed-edge descent ledgers.</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Superseded</x:v>
+        <x:v>Repair target</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
+        <x:v>Construct this readout/witness package for every bottleneck interval, or extract a normalized-law counterexample from a finite failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" t="str">
-        <x:v>Unit-continuation abelian-kernel lift</x:v>
+        <x:v>Superseded completion audit</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
+        <x:v>Keep the earlier internal completion checklist as historical context only.</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
+        <x:v>proofs/final_completion_audit.md is marked superseded by proofs/proof_critic_gap_audit.md.</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Reduction criterion</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
+        <x:v>Do not cite this file as outcome A without repairing the proof-critic gap.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" t="str">
-        <x:v>Unit-continuation derived series</x:v>
+        <x:v>Unit-continuation abelian-kernel lift</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
+        <x:v>Split the final unit endpoint into finite abelianization plus commutator-kernel correction.</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
+        <x:v>proofs/unit_continuation_abelian_kernel_lift.md; normal_quotient_longitude_lift_audit checks quotient witness, lifted witness, and kernel witness.</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
+        <x:v>Prove abelian matrix witnesses and commutator-kernel witnesses for S_beta in the fixed unit group.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" t="str">
-        <x:v>Bi-free subgroup certificate</x:v>
+        <x:v>Unit-continuation derived series</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
+        <x:v>Iterate the abelian-kernel split through the finite derived series of the fixed unit group.</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
+        <x:v>proofs/unit_continuation_derived_series_reduction.md; derived_series_audit records solvable collapse or the perfect residual.</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Reduction criterion</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
+        <x:v>Solvable unit groups reduce to abelian matrix witnesses; nonsolvable obstruction must live in the perfect residual.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" t="str">
-        <x:v>Bi-free certificate audit</x:v>
+        <x:v>Bi-free subgroup certificate</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
+        <x:v>Profile candidate words against fixed corridor detector factors.</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
+        <x:v>Helper, extra-factor target support, direct-product subgroup audit, and tests added; affine commutator seen by S3 block factor.</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Bounded audit</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
+        <x:v>Upgrade finite certificates to all-n factorization or law sequence.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" t="str">
-        <x:v>Bi-free exact audit</x:v>
+        <x:v>Bi-free certificate audit</x:v>
       </x:c>
       <x:c r="B113" t="str">
-        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
+        <x:v>Apply corridor certificate to local-minimal cover corpus.</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
+        <x:v>Size3: 116 product_finite_g, 12 nondegenerate, 6 known_total, 0 product/corridor targets.</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Bounded audit</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
+        <x:v>Prove arbitrary-fibre theorem or find normalized-law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" t="str">
-        <x:v>Kernel closure</x:v>
+        <x:v>Bi-free exact audit</x:v>
       </x:c>
       <x:c r="B114" t="str">
-        <x:v>Close coordinate kernels.</x:v>
+        <x:v>Close fixed-index image using the same corridor detector factor list.</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
+        <x:v>Affine stress row n=2: 12 states, no kernel/collision failure; product subgroup check matches factor product.</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
+        <x:v>Upgrade fixed-n closure to all-n corridor factorization.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="48" customHeight="1">
       <x:c r="A115" t="str">
-        <x:v>Kernel corridor</x:v>
+        <x:v>Kernel closure</x:v>
       </x:c>
       <x:c r="B115" t="str">
-        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
+        <x:v>Close coordinate kernels.</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
+        <x:v>Equality=nondegenerate; elementary kernel-pair closures must be universal in local-minimal degenerate rows.</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
+        <x:v>Control universal kernel-closure branch or refine nonminimal intervals.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="48" customHeight="1">
       <x:c r="A116" t="str">
-        <x:v>Universal corridor target</x:v>
+        <x:v>Kernel corridor</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>State remaining universal-kernel A/B branch.</x:v>
+        <x:v>Distinguish seed-only vs transported universal closures.</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Affine depth 1 rows are involutive.</x:v>
+        <x:v>Size&lt;=3: no semisplit leaks; LocalMasterBottleneckSummary now records elementary output-kernel pair counts/failures/depth.</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Open</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>Prove detector or find law escape.</x:v>
+        <x:v>Prove lemma or find normalized-law escape along universal pair corridors.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="48" customHeight="1">
       <x:c r="A117" t="str">
-        <x:v>Corridor-Green bridge</x:v>
+        <x:v>Universal corridor target</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
+        <x:v>State remaining universal-kernel A/B branch.</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
+        <x:v>Affine depth 1 rows are involutive.</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Candidate audit</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>Prove bridge symbolically.</x:v>
+        <x:v>Prove detector or find law escape.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="48" customHeight="1">
       <x:c r="A118" t="str">
-        <x:v>Product-permutation</x:v>
+        <x:v>Corridor-Green bridge</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Normalize swapped and direct universal branches.</x:v>
+        <x:v>Cross-tab universal corridors with Green hidden loops.</x:v>
       </x:c>
       <x:c r="C118" t="str">
-        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
+        <x:v>Size&lt;=3 overlap has 0 untagged intervals.</x:v>
       </x:c>
       <x:c r="D118" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Candidate audit</x:v>
       </x:c>
       <x:c r="E118" t="str">
-        <x:v>Prove H_prod words are longitude products.</x:v>
+        <x:v>Prove bridge symbolically.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="48" customHeight="1">
       <x:c r="A119" t="str">
-        <x:v>Swapped nondegenerate base</x:v>
+        <x:v>Product-permutation</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
+        <x:v>Normalize swapped and direct universal branches.</x:v>
       </x:c>
       <x:c r="C119" t="str">
-        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
+        <x:v>H_prod explicit; coboundaries telescope; closed product detector groups added to bottleneck summary.</x:v>
       </x:c>
       <x:c r="D119" t="str">
-        <x:v>Reduction ready</x:v>
+        <x:v>Executable audit</x:v>
       </x:c>
       <x:c r="E119" t="str">
-        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
+        <x:v>Prove H_prod words are longitude products.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="48" customHeight="1">
       <x:c r="A120" t="str">
-        <x:v>Identity-base product</x:v>
+        <x:v>Swapped nondegenerate base</x:v>
       </x:c>
       <x:c r="B120" t="str">
-        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
+        <x:v>Swapped product extension over nondegenerate quotient is nondegenerate.</x:v>
       </x:c>
       <x:c r="C120" t="str">
-        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
+        <x:v>All-n fibre-bijection proof added; regression fixture checks the known product row.</x:v>
       </x:c>
       <x:c r="D120" t="str">
         <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E120" t="str">
-        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
+        <x:v>Route such rows to the nondegenerate/guitar branch, not to product holonomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="48" customHeight="1">
       <x:c r="A121" t="str">
-        <x:v>Product closed labels</x:v>
+        <x:v>Identity-base product</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Closed product holonomy as finite labels.</x:v>
+        <x:v>Reduce identity-base product holonomy to swapped K_a or direct identities.</x:v>
       </x:c>
       <x:c r="C121" t="str">
-        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
+        <x:v>Central-label/direct-trivial reducers plus cyclic detector implemented.</x:v>
       </x:c>
       <x:c r="D121" t="str">
-        <x:v>Exact fixed-n audit</x:v>
+        <x:v>Reduction ready</x:v>
       </x:c>
       <x:c r="E121" t="str">
-        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
+        <x:v>Use as known product subbranch; obstruction needs non-identity colours.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="48" customHeight="1">
       <x:c r="A122" t="str">
-        <x:v>Product witnesses</x:v>
+        <x:v>Product closed labels</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Avoid false common-assignment shortcut.</x:v>
+        <x:v>Closed product holonomy as finite labels.</x:v>
       </x:c>
       <x:c r="C122" t="str">
-        <x:v>Route audit records common-assignment failure, per-label witnesses, and subgroup membership.</x:v>
+        <x:v>Exact n=2 all-base audit: 0 untagged failures; known-row miss fixed by S4 factor.</x:v>
       </x:c>
       <x:c r="D122" t="str">
-        <x:v>Executable audit</x:v>
+        <x:v>Exact fixed-n audit</x:v>
       </x:c>
       <x:c r="E122" t="str">
-        <x:v>Use only as route bookkeeping; prove subgroup condition symbolically.</x:v>
+        <x:v>Upgrade fixed-tuple certificates to all-n product lemma.</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="48" customHeight="1">
    